<commit_message>
P1 영역1: aiattack 구조 정합(v3)
- IM-03.1 크립토재킹·IM-03.2 LLMjacking(AI가 피해 대상) 삭제 → AI·클라우드 연계만(사용자 결정).
  관련 사고 AII-005·015 제외, AII-016은 측면 이동(AO-05)으로만 유지, ASN-08 시나리오 제거
- 통제 이탈 자율 에이전트 행 AIA-AO-06 신설(D14) — AII-010(OpenAI 평가→Hugging Face) 재매핑, OWASP ASI10
- 방어·연구 측 역량 실증(Big Sleep·XBOW) capability_indicator로 표시해 공격자 사고 집계 제외(D13)
- VE 도메인명 '취약점 발굴·익스플로잇·악성코드 생성'으로 확장(행 위치 유지, 사용자 결정)
- 결과: 세부위협 35→34, 사고 34→32, 시나리오 8→7, 위험도 매우높음 10·높음 8·보통 15·낮음 1
- 통합 v5 뷰 재생성, README·methodology·작업방향 갱신. AI 역할 2차원 분리는 후속 증분

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RuSCf1v2AwGLbjYwwieALL
</commit_message>
<xml_diff>
--- a/integrated/output/통합_보안위협_매트릭스_v5_AI활용공격뷰.xlsx
+++ b/integrated/output/통합_보안위협_매트릭스_v5_AI활용공격뷰.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="평가 기준·메모" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'AI 활용 공격 뷰'!$A$3:$J$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'렌즈 교차 매핑'!$A$3:$G$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'AI 활용 공격 뷰'!$A$3:$J$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'렌즈 교차 매핑'!$A$3:$G$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>통합 v4.1 기준 그대로 유지(변동 없음) — 뷰 레이어 35개는 고유 위협 수에 더하지 않음</t>
+          <t>통합 v4.1 기준 그대로 유지(변동 없음) — 뷰 레이어 34개는 고유 위협 수에 더하지 않음</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>35개(공격자 킬체인 7단계) — 위험도 매우 높음 10 · 높음 9 · 보통 15 · 낮음 1</t>
+          <t>34개(공격자 킬체인 7단계) — 위험도 매우 높음 10 · 높음 8 · 보통 15 · 낮음 1</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>기존 237개 중 28개를 AI 활용 공격 렌즈가 닿음(연계). 나머지는 이 렌즈 밖</t>
+          <t>기존 237개 중 25개를 AI 활용 공격 렌즈가 닿음(연계). 나머지는 이 렌즈 밖</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>AI 보안위협 12/60 · 클라우드 보안위협 4/38 · OT 보안위협 1/50 · 공급망 보안위협 4/30 · 신원 보안위협 6/32 · 물리·인적 보안위협 1/27</t>
+          <t>AI 보안위협 11/60 · 클라우드 보안위협 2/38 · OT 보안위협 1/50 · 공급망 보안위협 4/30 · 신원 보안위협 6/32 · 물리·인적 보안위협 1/27</t>
         </is>
       </c>
     </row>
@@ -744,7 +744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>16</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>15</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>13</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
@@ -1571,17 +1571,17 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>[IM] 영향·규모화</t>
+          <t>[VE] 취약점 발굴·익스플로잇 생성</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>AIA-IM-03.1</t>
+          <t>AIA-VE-01.1</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>AI 인프라 악용 크립토재킹</t>
+          <t>AI 자율 취약점 발굴(버그 헌팅)</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
@@ -1591,17 +1591,17 @@
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>17</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>보조</t>
+          <t>완전자율</t>
         </is>
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>증폭</t>
+          <t>신규</t>
         </is>
       </c>
       <c r="H19" s="9" t="inlineStr">
@@ -1609,13 +1609,9 @@
           <t>실사용</t>
         </is>
       </c>
-      <c r="I19" s="7" t="inlineStr">
-        <is>
-          <t>AI-09-03, CL-IM-06</t>
-        </is>
-      </c>
+      <c r="I19" s="7" t="inlineStr"/>
       <c r="J19" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -1626,12 +1622,12 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>AIA-VE-01.1</t>
+          <t>AIA-VE-02</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>AI 자율 취약점 발굴(버그 헌팅)</t>
+          <t>AI 익스플로잇 자동 생성·개발</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
@@ -1646,7 +1642,7 @@
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>완전자율</t>
+          <t>반자율</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
@@ -1672,12 +1668,12 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>AIA-VE-02</t>
+          <t>AIA-VE-03.2</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>AI 익스플로잇 자동 생성·개발</t>
+          <t>AI 생성 와이퍼·파괴 스크립트</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
@@ -1687,17 +1683,17 @@
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>14</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>반자율</t>
+          <t>보조</t>
         </is>
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>신규</t>
+          <t>증폭</t>
         </is>
       </c>
       <c r="H21" s="9" t="inlineStr">
@@ -1705,45 +1701,49 @@
           <t>실사용</t>
         </is>
       </c>
-      <c r="I21" s="7" t="inlineStr"/>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t>AI-01-06, OT-IR-01</t>
+        </is>
+      </c>
       <c r="J21" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>[VE] 취약점 발굴·익스플로잇 생성</t>
+          <t>[AO] 자율 실행·확산</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>AIA-VE-03.2</t>
+          <t>AIA-AO-06</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>AI 생성 와이퍼·파괴 스크립트</t>
-        </is>
-      </c>
-      <c r="D22" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+          <t>통제를 벗어난 자율 에이전트의 자발적 침해(사람 공격자 없음)</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>23</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>보조</t>
+          <t>완전자율</t>
         </is>
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>증폭</t>
+          <t>신규</t>
         </is>
       </c>
       <c r="H22" s="9" t="inlineStr">
@@ -1753,11 +1753,11 @@
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>AI-01-06, OT-IR-01</t>
+          <t>AI-01-05</t>
         </is>
       </c>
       <c r="J22" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>25</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>21</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>31</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>20</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>24</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
@@ -2018,12 +2018,12 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>AIA-IM-03.2</t>
+          <t>AIA-IM-04</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>LLMjacking·AI 과금 폭탄</t>
+          <t>AI 활용 공격의 규모화·대량화</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2033,17 +2033,17 @@
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>30</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>보조</t>
+          <t>반자율</t>
         </is>
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>신규</t>
+          <t>증폭</t>
         </is>
       </c>
       <c r="H28" s="9" t="inlineStr">
@@ -2053,27 +2053,27 @@
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>AI-09-02, CL-IM-07</t>
+          <t>AI-01-05</t>
         </is>
       </c>
       <c r="J28" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>[IM] 영향·규모화</t>
+          <t>[RD] 공격 역량 확보</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>AIA-IM-04</t>
+          <t>AIA-RD-01.1</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>AI 활용 공격의 규모화·대량화</t>
+          <t>다크 LLM·탈옥 모델 확보</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
@@ -2083,17 +2083,17 @@
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>28</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>반자율</t>
+          <t>보조</t>
         </is>
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>증폭</t>
+          <t>신규</t>
         </is>
       </c>
       <c r="H29" s="9" t="inlineStr">
@@ -2103,7 +2103,7 @@
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>AI-01-05</t>
+          <t>AI-01-03</t>
         </is>
       </c>
       <c r="J29" s="9" t="n">
@@ -2118,12 +2118,12 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>AIA-RD-01.1</t>
+          <t>AIA-RD-02</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>다크 LLM·탈옥 모델 확보</t>
+          <t>AI 기반 공격 도구·스크립트·셸 명령 생성</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2133,17 +2133,17 @@
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>26</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>보조</t>
+          <t>증강</t>
         </is>
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>신규</t>
+          <t>증폭</t>
         </is>
       </c>
       <c r="H30" s="9" t="inlineStr">
@@ -2168,12 +2168,12 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>AIA-RD-02</t>
+          <t>AIA-RD-03</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>AI 기반 공격 도구·스크립트·셸 명령 생성</t>
+          <t>공격 인프라·AI 서비스 프록시 확보</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr">
@@ -2183,12 +2183,12 @@
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>32</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>증강</t>
+          <t>보조</t>
         </is>
       </c>
       <c r="G31" s="9" t="inlineStr">
@@ -2198,32 +2198,32 @@
       </c>
       <c r="H31" s="9" t="inlineStr">
         <is>
-          <t>실사용</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="I31" s="7" t="inlineStr">
         <is>
-          <t>AI-01-03</t>
+          <t>AI-09-03, CL-RD-01</t>
         </is>
       </c>
       <c r="J31" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>[RD] 공격 역량 확보</t>
+          <t>[RT] 정찰·표적 분석</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>AIA-RD-03</t>
+          <t>AIA-RT-01.1</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>공격 인프라·AI 서비스 프록시 확보</t>
+          <t>AI 기반 공개정보 수집·인물 프로파일링</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2233,12 +2233,12 @@
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>27</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>보조</t>
+          <t>증강</t>
         </is>
       </c>
       <c r="G32" s="9" t="inlineStr">
@@ -2248,12 +2248,12 @@
       </c>
       <c r="H32" s="9" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>실사용</t>
         </is>
       </c>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t>AI-09-03, CL-RD-01</t>
+          <t>AI-01-01, PH-RC-01</t>
         </is>
       </c>
       <c r="J32" s="9" t="n">
@@ -2268,12 +2268,12 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>AIA-RT-01.1</t>
+          <t>AIA-RT-01.2</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>AI 기반 공개정보 수집·인물 프로파일링</t>
+          <t>AI 기반 표적 환경·관계 분석</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
@@ -2298,16 +2298,16 @@
       </c>
       <c r="H33" s="9" t="inlineStr">
         <is>
-          <t>실사용</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="I33" s="7" t="inlineStr">
         <is>
-          <t>AI-01-01, PH-RC-01</t>
+          <t>AI-01-01</t>
         </is>
       </c>
       <c r="J33" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -2318,12 +2318,12 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>AIA-RT-01.2</t>
+          <t>AIA-RT-02</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>AI 기반 표적 환경·관계 분석</t>
+          <t>AI 에이전트의 노출 자산·공격면 자동 식별</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2333,12 +2333,12 @@
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>19</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>증강</t>
+          <t>반자율</t>
         </is>
       </c>
       <c r="G34" s="9" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="H34" s="9" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>실사용</t>
         </is>
       </c>
       <c r="I34" s="7" t="inlineStr">
@@ -2368,12 +2368,12 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>AIA-RT-02</t>
+          <t>AIA-RT-03</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>AI 에이전트의 노출 자산·공격면 자동 식별</t>
+          <t>AI 기반 취약점 정보·공개 PoC 자동 수집·분류</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
@@ -2383,12 +2383,12 @@
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>반자율</t>
+          <t>증강</t>
         </is>
       </c>
       <c r="G35" s="9" t="inlineStr">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="I35" s="7" t="inlineStr">
         <is>
-          <t>AI-01-01</t>
+          <t>AI-01-03</t>
         </is>
       </c>
       <c r="J35" s="9" t="n">
@@ -2413,17 +2413,17 @@
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>[RT] 정찰·표적 분석</t>
+          <t>[VE] 취약점 발굴·익스플로잇 생성</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>AIA-RT-03</t>
+          <t>AIA-VE-01.2</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>AI 기반 취약점 정보·공개 PoC 자동 수집·분류</t>
+          <t>AI 보조 코드 감사·퍼징</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>33</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
@@ -2448,12 +2448,12 @@
       </c>
       <c r="H36" s="9" t="inlineStr">
         <is>
-          <t>실사용</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="I36" s="7" t="inlineStr">
         <is>
-          <t>AI-01-03</t>
+          <t>SC-DP-04</t>
         </is>
       </c>
       <c r="J36" s="9" t="n">
@@ -2463,22 +2463,22 @@
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>[VE] 취약점 발굴·익스플로잇 생성</t>
+          <t>[RD] 공격 역량 확보</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>AIA-VE-01.2</t>
+          <t>AIA-RD-01.2</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>AI 보조 코드 감사·퍼징</t>
-        </is>
-      </c>
-      <c r="D37" s="11" t="inlineStr">
-        <is>
-          <t>보통</t>
+          <t>증류·파인튜닝으로 공세 역량 확보</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>낮음</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
@@ -2488,80 +2488,30 @@
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>증강</t>
+          <t>보조</t>
         </is>
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>증폭</t>
+          <t>신규</t>
         </is>
       </c>
       <c r="H37" s="9" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>연구시연</t>
         </is>
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
-          <t>SC-DP-04</t>
+          <t>AI-01-03</t>
         </is>
       </c>
       <c r="J37" s="9" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="7" t="inlineStr">
-        <is>
-          <t>[RD] 공격 역량 확보</t>
-        </is>
-      </c>
-      <c r="B38" s="7" t="inlineStr">
-        <is>
-          <t>AIA-RD-01.2</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>증류·파인튜닝으로 공세 역량 확보</t>
-        </is>
-      </c>
-      <c r="D38" s="12" t="inlineStr">
-        <is>
-          <t>낮음</t>
-        </is>
-      </c>
-      <c r="E38" s="9" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="F38" s="9" t="inlineStr">
-        <is>
-          <t>보조</t>
-        </is>
-      </c>
-      <c r="G38" s="9" t="inlineStr">
-        <is>
-          <t>신규</t>
-        </is>
-      </c>
-      <c r="H38" s="9" t="inlineStr">
-        <is>
-          <t>연구시연</t>
-        </is>
-      </c>
-      <c r="I38" s="7" t="inlineStr">
-        <is>
-          <t>AI-01-03</t>
-        </is>
-      </c>
-      <c r="J38" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A3:J38"/>
+  <autoFilter ref="A3:J37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2572,7 +2522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3038,17 +2988,17 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>AIA-CC-01</t>
+          <t>AIA-AO-06</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>AI 서비스 API·웹 인터페이스 경유 은닉 C2</t>
-        </is>
-      </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+          <t>통제를 벗어난 자율 에이전트의 자발적 침해(사람 공격자 없음)</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -3058,12 +3008,12 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>AI-01-09</t>
+          <t>AI-01-05</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>AI 서비스 경유 은닉 C2</t>
+          <t>자율·다중 에이전트 기반 공격</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
@@ -3075,12 +3025,12 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>AIA-CC-02</t>
+          <t>AIA-CC-01</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>실행 중 AI 명령 동적 생성 악성코드</t>
+          <t>AI 서비스 API·웹 인터페이스 경유 은닉 C2</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
@@ -3095,12 +3045,12 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>AI-01-06</t>
+          <t>AI-01-09</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>AI 연동 악성코드</t>
+          <t>AI 서비스 경유 은닉 C2</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr">
@@ -3112,17 +3062,17 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>AIA-CC-03</t>
+          <t>AIA-CC-02</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>AI 기반 방어 회피·난독화</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>보통</t>
+          <t>실행 중 AI 명령 동적 생성 악성코드</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>높음</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -3132,29 +3082,29 @@
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>AI-04-04</t>
+          <t>AI-01-06</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>적대적 입력 기반 판단 회피</t>
-        </is>
-      </c>
-      <c r="G17" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+          <t>AI 연동 악성코드</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>매우 높음</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>AIA-CC-04</t>
+          <t>AIA-CC-03</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>AI 코딩 도구 규칙·설정 숨은 지시 주입</t>
+          <t>AI 기반 방어 회피·난독화</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
@@ -3169,17 +3119,17 @@
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>AI-08-05</t>
+          <t>AI-04-04</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>악성 에이전트 도구 유통과 AI 코딩 도구 오염</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>매우 높음</t>
+          <t>적대적 입력 기반 판단 회피</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>높음</t>
         </is>
       </c>
     </row>
@@ -3201,17 +3151,17 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>공급망 보안위협</t>
+          <t>AI 보안위협</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>SC-DE-02</t>
+          <t>AI-08-05</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>IDE 확장·개발 도구·툴체인 오염</t>
+          <t>악성 에이전트 도구 유통과 AI 코딩 도구 오염</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
@@ -3223,37 +3173,37 @@
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>AIA-IA-01.1</t>
+          <t>AIA-CC-04</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>AI 생성 대량 피싱·미끼</t>
-        </is>
-      </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+          <t>AI 코딩 도구 규칙·설정 숨은 지시 주입</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>AI 보안위협</t>
+          <t>공급망 보안위협</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>AI-01-08</t>
+          <t>SC-DE-02</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>AI 생성 피싱 및 신뢰 주체 사칭</t>
-        </is>
-      </c>
-      <c r="G20" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+          <t>IDE 확장·개발 도구·툴체인 오염</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>매우 높음</t>
         </is>
       </c>
     </row>
@@ -3275,17 +3225,17 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>신원 보안위협</t>
+          <t>AI 보안위협</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>ID-SE-01</t>
+          <t>AI-01-08</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>인증 피싱(AiTM·OAuth 동의·문자·메신저)</t>
+          <t>AI 생성 피싱 및 신뢰 주체 사칭</t>
         </is>
       </c>
       <c r="G21" s="10" t="inlineStr">
@@ -3297,32 +3247,32 @@
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>AIA-IA-01.2</t>
+          <t>AIA-IA-01.1</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>AI 기반 표적 스피어피싱·BEC</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="inlineStr">
-        <is>
-          <t>보통</t>
+          <t>AI 생성 대량 피싱·미끼</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>높음</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>AI 보안위협</t>
+          <t>신원 보안위협</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>AI-01-08</t>
+          <t>ID-SE-01</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>AI 생성 피싱 및 신뢰 주체 사칭</t>
+          <t>인증 피싱(AiTM·OAuth 동의·문자·메신저)</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr">
@@ -3349,17 +3299,17 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>신원 보안위협</t>
+          <t>AI 보안위협</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>ID-SE-01</t>
+          <t>AI-01-08</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>인증 피싱(AiTM·OAuth 동의·문자·메신저)</t>
+          <t>AI 생성 피싱 및 신뢰 주체 사칭</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">
@@ -3371,32 +3321,32 @@
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>AIA-IA-02.1</t>
+          <t>AIA-IA-01.2</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>영상 딥페이크 사칭</t>
-        </is>
-      </c>
-      <c r="C24" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+          <t>AI 기반 표적 스피어피싱·BEC</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>AI 보안위협</t>
+          <t>신원 보안위협</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>AI-01-08</t>
+          <t>ID-SE-01</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>AI 생성 피싱 및 신뢰 주체 사칭</t>
+          <t>인증 피싱(AiTM·OAuth 동의·문자·메신저)</t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr">
@@ -3423,17 +3373,17 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>신원 보안위협</t>
+          <t>AI 보안위협</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>ID-SE-04</t>
+          <t>AI-01-08</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>딥페이크·AI 음성 사칭(송금·접근 요청)</t>
+          <t>AI 생성 피싱 및 신뢰 주체 사칭</t>
         </is>
       </c>
       <c r="G25" s="10" t="inlineStr">
@@ -3445,32 +3395,32 @@
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>AIA-IA-02.2</t>
+          <t>AIA-IA-02.1</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>음성 딥페이크 사칭</t>
-        </is>
-      </c>
-      <c r="C26" s="11" t="inlineStr">
-        <is>
-          <t>보통</t>
+          <t>영상 딥페이크 사칭</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>높음</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>AI 보안위협</t>
+          <t>신원 보안위협</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>AI-01-08</t>
+          <t>ID-SE-04</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>AI 생성 피싱 및 신뢰 주체 사칭</t>
+          <t>딥페이크·AI 음성 사칭(송금·접근 요청)</t>
         </is>
       </c>
       <c r="G26" s="10" t="inlineStr">
@@ -3497,17 +3447,17 @@
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>신원 보안위협</t>
+          <t>AI 보안위협</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>ID-SE-04</t>
+          <t>AI-01-08</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>딥페이크·AI 음성 사칭(송금·접근 요청)</t>
+          <t>AI 생성 피싱 및 신뢰 주체 사칭</t>
         </is>
       </c>
       <c r="G27" s="10" t="inlineStr">
@@ -3519,32 +3469,32 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>AIA-IA-03</t>
+          <t>AIA-IA-02.2</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>딥페이크 기반 생체·본인확인 우회</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>매우 높음</t>
+          <t>음성 딥페이크 사칭</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>AI 보안위협</t>
+          <t>신원 보안위협</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>AI-01-08</t>
+          <t>ID-SE-04</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>AI 생성 피싱 및 신뢰 주체 사칭</t>
+          <t>딥페이크·AI 음성 사칭(송금·접근 요청)</t>
         </is>
       </c>
       <c r="G28" s="10" t="inlineStr">
@@ -3571,17 +3521,17 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>신원 보안위협</t>
+          <t>AI 보안위협</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>ID-CI-03</t>
+          <t>AI-01-08</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>명의 도용·본인확인 우회(딥페이크 포함)</t>
+          <t>AI 생성 피싱 및 신뢰 주체 사칭</t>
         </is>
       </c>
       <c r="G29" s="10" t="inlineStr">
@@ -3593,32 +3543,32 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>AIA-IA-04</t>
+          <t>AIA-IA-03</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>AI 미끼·ClickFix·크래프트 링크로 실행 유도</t>
-        </is>
-      </c>
-      <c r="C30" s="11" t="inlineStr">
-        <is>
-          <t>보통</t>
+          <t>딥페이크 기반 생체·본인확인 우회</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>매우 높음</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>AI 보안위협</t>
+          <t>신원 보안위협</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>AI-01-08</t>
+          <t>ID-CI-03</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>AI 생성 피싱 및 신뢰 주체 사칭</t>
+          <t>명의 도용·본인확인 우회(딥페이크 포함)</t>
         </is>
       </c>
       <c r="G30" s="10" t="inlineStr">
@@ -3630,17 +3580,17 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>AIA-IM-01</t>
+          <t>AIA-IA-04</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>딥페이크·AI 사칭 기반 금전 사기</t>
-        </is>
-      </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+          <t>AI 미끼·ClickFix·크래프트 링크로 실행 유도</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
@@ -3682,54 +3632,54 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>신원 보안위협</t>
+          <t>AI 보안위협</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>ID-IM-01</t>
+          <t>AI-01-08</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>계정 장악 기반 금전 사기(BEC·송금·사칭 게시)</t>
-        </is>
-      </c>
-      <c r="G32" s="8" t="inlineStr">
-        <is>
-          <t>매우 높음</t>
+          <t>AI 생성 피싱 및 신뢰 주체 사칭</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="inlineStr">
+        <is>
+          <t>높음</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>AIA-IM-02</t>
+          <t>AIA-IM-01</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>AI 가속 대규모 데이터 탈취·반출</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>매우 높음</t>
+          <t>딥페이크·AI 사칭 기반 금전 사기</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>높음</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>AI 보안위협</t>
+          <t>신원 보안위협</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>AI-01-05</t>
+          <t>ID-IM-01</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>자율·다중 에이전트 기반 공격</t>
+          <t>계정 장악 기반 금전 사기(BEC·송금·사칭 게시)</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr">
@@ -3756,17 +3706,17 @@
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>신원 보안위협</t>
+          <t>AI 보안위협</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>ID-IM-03</t>
+          <t>AI-01-05</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>계정 기반 대량 데이터 탈취·갈취</t>
+          <t>자율·다중 에이전트 기반 공격</t>
         </is>
       </c>
       <c r="G34" s="8" t="inlineStr">
@@ -3778,32 +3728,32 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>AIA-IM-03.1</t>
+          <t>AIA-IM-02</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>AI 인프라 악용 크립토재킹</t>
-        </is>
-      </c>
-      <c r="C35" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+          <t>AI 가속 대규모 데이터 탈취·반출</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>매우 높음</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>AI 보안위협</t>
+          <t>신원 보안위협</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>AI-09-03</t>
+          <t>ID-IM-03</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>외부 노출 AI 서비스</t>
+          <t>계정 기반 대량 데이터 탈취·갈취</t>
         </is>
       </c>
       <c r="G35" s="8" t="inlineStr">
@@ -3815,32 +3765,32 @@
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>AIA-IM-03.1</t>
+          <t>AIA-IM-04</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>AI 인프라 악용 크립토재킹</t>
-        </is>
-      </c>
-      <c r="C36" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+          <t>AI 활용 공격의 규모화·대량화</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>클라우드 보안위협</t>
+          <t>AI 보안위협</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>CL-IM-06</t>
+          <t>AI-01-05</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>컴퓨팅 자원 탈취(크립토재킹)</t>
+          <t>자율·다중 에이전트 기반 공격</t>
         </is>
       </c>
       <c r="G36" s="8" t="inlineStr">
@@ -3852,12 +3802,12 @@
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>AIA-IM-03.2</t>
+          <t>AIA-RD-01.1</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>LLMjacking·AI 과금 폭탄</t>
+          <t>다크 LLM·탈옥 모델 확보</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
@@ -3872,12 +3822,12 @@
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>AI-09-02</t>
+          <t>AI-01-03</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>AI 과금 폭탄 및 에이전트 루프 소모</t>
+          <t>공격 도구·인프라 및 AI 자원 확보</t>
         </is>
       </c>
       <c r="G37" s="11" t="inlineStr">
@@ -3889,49 +3839,49 @@
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>AIA-IM-03.2</t>
+          <t>AIA-RD-01.2</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>LLMjacking·AI 과금 폭탄</t>
-        </is>
-      </c>
-      <c r="C38" s="11" t="inlineStr">
+          <t>증류·파인튜닝으로 공세 역량 확보</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>낮음</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>AI 보안위협</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>AI-01-03</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>공격 도구·인프라 및 AI 자원 확보</t>
+        </is>
+      </c>
+      <c r="G38" s="11" t="inlineStr">
         <is>
           <t>보통</t>
-        </is>
-      </c>
-      <c r="D38" s="7" t="inlineStr">
-        <is>
-          <t>클라우드 보안위협</t>
-        </is>
-      </c>
-      <c r="E38" s="7" t="inlineStr">
-        <is>
-          <t>CL-IM-07</t>
-        </is>
-      </c>
-      <c r="F38" s="7" t="inlineStr">
-        <is>
-          <t>관리형 서비스 악용(LLMjacking·SMS 펌핑)</t>
-        </is>
-      </c>
-      <c r="G38" s="8" t="inlineStr">
-        <is>
-          <t>매우 높음</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>AIA-IM-04</t>
+          <t>AIA-RD-02</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>AI 활용 공격의 규모화·대량화</t>
+          <t>AI 기반 공격 도구·스크립트·셸 명령 생성</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
@@ -3946,29 +3896,29 @@
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>AI-01-05</t>
+          <t>AI-01-03</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>자율·다중 에이전트 기반 공격</t>
-        </is>
-      </c>
-      <c r="G39" s="8" t="inlineStr">
-        <is>
-          <t>매우 높음</t>
+          <t>공격 도구·인프라 및 AI 자원 확보</t>
+        </is>
+      </c>
+      <c r="G39" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>AIA-RD-01.1</t>
+          <t>AIA-RD-03</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>다크 LLM·탈옥 모델 확보</t>
+          <t>공격 인프라·AI 서비스 프록시 확보</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
@@ -3983,49 +3933,49 @@
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>AI-01-03</t>
+          <t>AI-09-03</t>
         </is>
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>공격 도구·인프라 및 AI 자원 확보</t>
-        </is>
-      </c>
-      <c r="G40" s="11" t="inlineStr">
-        <is>
-          <t>보통</t>
+          <t>외부 노출 AI 서비스</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>매우 높음</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>AIA-RD-01.2</t>
+          <t>AIA-RD-03</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>증류·파인튜닝으로 공세 역량 확보</t>
-        </is>
-      </c>
-      <c r="C41" s="12" t="inlineStr">
-        <is>
-          <t>낮음</t>
+          <t>공격 인프라·AI 서비스 프록시 확보</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>AI 보안위협</t>
+          <t>클라우드 보안위협</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>AI-01-03</t>
+          <t>CL-RD-01</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>공격 도구·인프라 및 AI 자원 확보</t>
+          <t>공격 인프라 확보(유사 도메인·클라우드 서버)</t>
         </is>
       </c>
       <c r="G41" s="11" t="inlineStr">
@@ -4037,17 +3987,17 @@
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>AIA-RD-02</t>
+          <t>AIA-RD-04</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>AI 기반 공격 도구·스크립트·셸 명령 생성</t>
-        </is>
-      </c>
-      <c r="C42" s="11" t="inlineStr">
-        <is>
-          <t>보통</t>
+          <t>공세 AI 에이전트·공격 하네스 구축</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>매우 높음</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
@@ -4057,29 +4007,29 @@
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>AI-01-03</t>
+          <t>AI-01-05</t>
         </is>
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>공격 도구·인프라 및 AI 자원 확보</t>
-        </is>
-      </c>
-      <c r="G42" s="11" t="inlineStr">
-        <is>
-          <t>보통</t>
+          <t>자율·다중 에이전트 기반 공격</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>매우 높음</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>AIA-RD-03</t>
+          <t>AIA-RT-01.1</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>공격 인프라·AI 서비스 프록시 확보</t>
+          <t>AI 기반 공개정보 수집·인물 프로파일링</t>
         </is>
       </c>
       <c r="C43" s="11" t="inlineStr">
@@ -4094,29 +4044,29 @@
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>AI-09-03</t>
+          <t>AI-01-01</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>외부 노출 AI 서비스</t>
-        </is>
-      </c>
-      <c r="G43" s="8" t="inlineStr">
-        <is>
-          <t>매우 높음</t>
+          <t>AI 대상 정찰 및 노출 자산 식별</t>
+        </is>
+      </c>
+      <c r="G43" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>AIA-RD-03</t>
+          <t>AIA-RT-01.1</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>공격 인프라·AI 서비스 프록시 확보</t>
+          <t>AI 기반 공개정보 수집·인물 프로파일링</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
@@ -4126,39 +4076,39 @@
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>클라우드 보안위협</t>
+          <t>물리·인적 보안위협</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>CL-RD-01</t>
+          <t>PH-RC-01</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>공격 인프라 확보(유사 도메인·클라우드 서버)</t>
-        </is>
-      </c>
-      <c r="G44" s="11" t="inlineStr">
-        <is>
-          <t>보통</t>
+          <t>공개정보 기반 핵심 인력·시설 파악</t>
+        </is>
+      </c>
+      <c r="G44" s="10" t="inlineStr">
+        <is>
+          <t>높음</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>AIA-RD-04</t>
+          <t>AIA-RT-01.2</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>공세 AI 에이전트·공격 하네스 구축</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>매우 높음</t>
+          <t>AI 기반 표적 환경·관계 분석</t>
+        </is>
+      </c>
+      <c r="C45" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
@@ -4168,29 +4118,29 @@
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>AI-01-05</t>
+          <t>AI-01-01</t>
         </is>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>자율·다중 에이전트 기반 공격</t>
-        </is>
-      </c>
-      <c r="G45" s="8" t="inlineStr">
-        <is>
-          <t>매우 높음</t>
+          <t>AI 대상 정찰 및 노출 자산 식별</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>AIA-RT-01.1</t>
+          <t>AIA-RT-02</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>AI 기반 공개정보 수집·인물 프로파일링</t>
+          <t>AI 에이전트의 노출 자산·공격면 자동 식별</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
@@ -4222,12 +4172,12 @@
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>AIA-RT-01.1</t>
+          <t>AIA-RT-03</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>AI 기반 공개정보 수집·인물 프로파일링</t>
+          <t>AI 기반 취약점 정보·공개 PoC 자동 수집·분류</t>
         </is>
       </c>
       <c r="C47" s="11" t="inlineStr">
@@ -4237,34 +4187,34 @@
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>물리·인적 보안위협</t>
+          <t>AI 보안위협</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>PH-RC-01</t>
+          <t>AI-01-03</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>공개정보 기반 핵심 인력·시설 파악</t>
-        </is>
-      </c>
-      <c r="G47" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+          <t>공격 도구·인프라 및 AI 자원 확보</t>
+        </is>
+      </c>
+      <c r="G47" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>AIA-RT-01.2</t>
+          <t>AIA-VE-01.2</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>AI 기반 표적 환경·관계 분석</t>
+          <t>AI 보조 코드 감사·퍼징</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
@@ -4274,39 +4224,39 @@
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>AI 보안위협</t>
+          <t>공급망 보안위협</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>AI-01-01</t>
+          <t>SC-DP-04</t>
         </is>
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>AI 대상 정찰 및 노출 자산 식별</t>
-        </is>
-      </c>
-      <c r="G48" s="11" t="inlineStr">
-        <is>
-          <t>보통</t>
+          <t>알려진 취약점이 있는 구성요소 사용</t>
+        </is>
+      </c>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>매우 높음</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>AIA-RT-02</t>
+          <t>AIA-VE-03.1</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>AI 에이전트의 노출 자산·공격면 자동 식별</t>
-        </is>
-      </c>
-      <c r="C49" s="11" t="inlineStr">
-        <is>
-          <t>보통</t>
+          <t>AI 생성·AI 연동 악성코드</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>매우 높음</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
@@ -4316,34 +4266,34 @@
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>AI-01-01</t>
+          <t>AI-01-06</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>AI 대상 정찰 및 노출 자산 식별</t>
-        </is>
-      </c>
-      <c r="G49" s="11" t="inlineStr">
-        <is>
-          <t>보통</t>
+          <t>AI 연동 악성코드</t>
+        </is>
+      </c>
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t>매우 높음</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>AIA-RT-03</t>
+          <t>AIA-VE-03.2</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>AI 기반 취약점 정보·공개 PoC 자동 수집·분류</t>
-        </is>
-      </c>
-      <c r="C50" s="11" t="inlineStr">
-        <is>
-          <t>보통</t>
+          <t>AI 생성 와이퍼·파괴 스크립트</t>
+        </is>
+      </c>
+      <c r="C50" s="10" t="inlineStr">
+        <is>
+          <t>높음</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
@@ -4353,49 +4303,49 @@
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>AI-01-03</t>
+          <t>AI-01-06</t>
         </is>
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>공격 도구·인프라 및 AI 자원 확보</t>
-        </is>
-      </c>
-      <c r="G50" s="11" t="inlineStr">
-        <is>
-          <t>보통</t>
+          <t>AI 연동 악성코드</t>
+        </is>
+      </c>
+      <c r="G50" s="8" t="inlineStr">
+        <is>
+          <t>매우 높음</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>AIA-VE-01.2</t>
+          <t>AIA-VE-03.2</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>AI 보조 코드 감사·퍼징</t>
-        </is>
-      </c>
-      <c r="C51" s="11" t="inlineStr">
-        <is>
-          <t>보통</t>
+          <t>AI 생성 와이퍼·파괴 스크립트</t>
+        </is>
+      </c>
+      <c r="C51" s="10" t="inlineStr">
+        <is>
+          <t>높음</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>공급망 보안위협</t>
+          <t>OT 보안위협</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>SC-DP-04</t>
+          <t>OT-IR-01</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>알려진 취약점이 있는 구성요소 사용</t>
+          <t>데이터 파괴(와이퍼)</t>
         </is>
       </c>
       <c r="G51" s="8" t="inlineStr">
@@ -4404,119 +4354,8 @@
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="7" t="inlineStr">
-        <is>
-          <t>AIA-VE-03.1</t>
-        </is>
-      </c>
-      <c r="B52" s="7" t="inlineStr">
-        <is>
-          <t>AI 생성·AI 연동 악성코드</t>
-        </is>
-      </c>
-      <c r="C52" s="8" t="inlineStr">
-        <is>
-          <t>매우 높음</t>
-        </is>
-      </c>
-      <c r="D52" s="7" t="inlineStr">
-        <is>
-          <t>AI 보안위협</t>
-        </is>
-      </c>
-      <c r="E52" s="7" t="inlineStr">
-        <is>
-          <t>AI-01-06</t>
-        </is>
-      </c>
-      <c r="F52" s="7" t="inlineStr">
-        <is>
-          <t>AI 연동 악성코드</t>
-        </is>
-      </c>
-      <c r="G52" s="8" t="inlineStr">
-        <is>
-          <t>매우 높음</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="7" t="inlineStr">
-        <is>
-          <t>AIA-VE-03.2</t>
-        </is>
-      </c>
-      <c r="B53" s="7" t="inlineStr">
-        <is>
-          <t>AI 생성 와이퍼·파괴 스크립트</t>
-        </is>
-      </c>
-      <c r="C53" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
-        </is>
-      </c>
-      <c r="D53" s="7" t="inlineStr">
-        <is>
-          <t>AI 보안위협</t>
-        </is>
-      </c>
-      <c r="E53" s="7" t="inlineStr">
-        <is>
-          <t>AI-01-06</t>
-        </is>
-      </c>
-      <c r="F53" s="7" t="inlineStr">
-        <is>
-          <t>AI 연동 악성코드</t>
-        </is>
-      </c>
-      <c r="G53" s="8" t="inlineStr">
-        <is>
-          <t>매우 높음</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="7" t="inlineStr">
-        <is>
-          <t>AIA-VE-03.2</t>
-        </is>
-      </c>
-      <c r="B54" s="7" t="inlineStr">
-        <is>
-          <t>AI 생성 와이퍼·파괴 스크립트</t>
-        </is>
-      </c>
-      <c r="C54" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
-        </is>
-      </c>
-      <c r="D54" s="7" t="inlineStr">
-        <is>
-          <t>OT 보안위협</t>
-        </is>
-      </c>
-      <c r="E54" s="7" t="inlineStr">
-        <is>
-          <t>OT-IR-01</t>
-        </is>
-      </c>
-      <c r="F54" s="7" t="inlineStr">
-        <is>
-          <t>데이터 파괴(와이퍼)</t>
-        </is>
-      </c>
-      <c r="G54" s="8" t="inlineStr">
-        <is>
-          <t>매우 높음</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A3:G54"/>
+  <autoFilter ref="A3:G51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4581,14 +4420,14 @@
         <v>60</v>
       </c>
       <c r="C4" s="9" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D4" s="9" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>AI-01-01, AI-01-03, AI-01-05, AI-01-06, AI-01-08, AI-01-09, AI-04-04, AI-06-04, AI-08-05, AI-09-02, AI-09-03, AI-09-05</t>
+          <t>AI-01-01, AI-01-03, AI-01-05, AI-01-06, AI-01-08, AI-01-09, AI-04-04, AI-06-04, AI-08-05, AI-09-03, AI-09-05</t>
         </is>
       </c>
     </row>
@@ -4602,14 +4441,14 @@
         <v>38</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>CL-CA-06, CL-IM-06, CL-IM-07, CL-RD-01</t>
+          <t>CL-CA-06, CL-RD-01</t>
         </is>
       </c>
     </row>
@@ -4707,10 +4546,10 @@
         <v>237</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E10" s="7" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
P3 영역1: aiattack 평가 규칙 개정(v3)
검토 6.1 렌즈 매트릭스 보조 규칙:
- 심각도 영향만으로 판정(속도·규모·탐지 난이도 → 고유 축·우선순위). 역량 확보·발굴·생성·은닉·C2(RD·VE·CC) 행을 중으로 재조정, severity_rule·검증기 가드 반영
- 발생가능성 상 = 실제 사고 가중 2 이상 + 서로 다른 행위자·캠페인 2개 이상(확인 1·추정 0.5), 하 = 공격자 사용 1차 근거 없음 + 성숙도 연구시연
- ATLAS 사례는 'AI 피해 대상'이 대부분이라 발생가능성 독립 신호에서 제외(참고 열로만)
- 경계 플래그(실제 사고 1건 빼면 등급 하락하는 행)·성숙도 자동 산출 신설, 보고서용/통합/CSV에 경계 열 추가
- 결과: 위험도 매우높음 8·높음 4·보통 21·낮음 1, 발생가능성 상 10·중 23·하 1, 경계 7행
- 통합 v5 뷰·changelog·methodology·README 갱신

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RuSCf1v2AwGLbjYwwieALL
</commit_message>
<xml_diff>
--- a/integrated/output/통합_보안위협_매트릭스_v5_AI활용공격뷰.xlsx
+++ b/integrated/output/통합_보안위협_매트릭스_v5_AI활용공격뷰.xlsx
@@ -597,7 +597,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>34개(공격자 킬체인 7단계) — 위험도 매우 높음 10 · 높음 8 · 보통 15 · 낮음 1</t>
+          <t>34개(공격자 킬체인 7단계) — 위험도 매우 높음 8 · 높음 4 · 보통 21 · 낮음 1</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F7" s="9" t="inlineStr">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
@@ -1221,37 +1221,37 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>[RD] 공격 역량 확보</t>
+          <t>[IA] 초기 침투·사회공학</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>AIA-RD-04</t>
+          <t>AIA-IA-02.1</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>공세 AI 에이전트·공격 하네스 구축</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>매우 높음</t>
+          <t>영상 딥페이크 사칭</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>높음</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>반자율</t>
+          <t>보조</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>신규</t>
+          <t>증폭</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
@@ -1261,37 +1261,37 @@
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>AI-01-05</t>
+          <t>AI-01-08, ID-SE-04</t>
         </is>
       </c>
       <c r="J12" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>[VE] 취약점 발굴·익스플로잇 생성</t>
+          <t>[IM] 영향·규모화</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>AIA-VE-03.1</t>
+          <t>AIA-IM-01</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>AI 생성·AI 연동 악성코드</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>매우 높음</t>
+          <t>딥페이크·AI 사칭 기반 금전 사기</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>높음</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>11</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
@@ -1311,27 +1311,27 @@
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>AI-01-06</t>
+          <t>AI-01-08, ID-IM-01</t>
         </is>
       </c>
       <c r="J13" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>[CC] 은닉·명령제어</t>
+          <t>[RD] 공격 역량 확보</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>AIA-CC-01</t>
+          <t>AIA-RD-04</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>AI 서비스 API·웹 인터페이스 경유 은닉 C2</t>
+          <t>공세 AI 에이전트·공격 하네스 구축</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
@@ -1341,12 +1341,12 @@
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>보조</t>
+          <t>반자율</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>AI-01-09</t>
+          <t>AI-01-05</t>
         </is>
       </c>
       <c r="J14" s="9" t="n">
@@ -1371,17 +1371,17 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>[CC] 은닉·명령제어</t>
+          <t>[VE] 취약점 발굴·익스플로잇 생성</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>AIA-CC-02</t>
+          <t>AIA-VE-03.1</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>실행 중 AI 명령 동적 생성 악성코드</t>
+          <t>AI 생성·AI 연동 악성코드</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
@@ -1391,17 +1391,17 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>반자율</t>
+          <t>보조</t>
         </is>
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>신규</t>
+          <t>증폭</t>
         </is>
       </c>
       <c r="H15" s="9" t="inlineStr">
@@ -1421,37 +1421,37 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>[IA] 초기 침투·사회공학</t>
+          <t>[AO] 자율 실행·확산</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>AIA-IA-01.1</t>
+          <t>AIA-AO-06</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>AI 생성 대량 피싱·미끼</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+          <t>통제를 벗어난 자율 에이전트의 자발적 침해(사람 공격자 없음)</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>19</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>보조</t>
+          <t>완전자율</t>
         </is>
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>증폭</t>
+          <t>신규</t>
         </is>
       </c>
       <c r="H16" s="9" t="inlineStr">
@@ -1461,37 +1461,37 @@
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>AI-01-08, ID-SE-01</t>
+          <t>AI-01-05</t>
         </is>
       </c>
       <c r="J16" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>[IA] 초기 침투·사회공학</t>
+          <t>[CC] 은닉·명령제어</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>AIA-IA-02.1</t>
+          <t>AIA-CC-01</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>영상 딥페이크 사칭</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+          <t>AI 서비스 API·웹 인터페이스 경유 은닉 C2</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>21</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
@@ -1501,7 +1501,7 @@
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>증폭</t>
+          <t>신규</t>
         </is>
       </c>
       <c r="H17" s="9" t="inlineStr">
@@ -1511,47 +1511,47 @@
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>AI-01-08, ID-SE-04</t>
+          <t>AI-01-09</t>
         </is>
       </c>
       <c r="J17" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>[IM] 영향·규모화</t>
+          <t>[CC] 은닉·명령제어</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>AIA-IM-01</t>
+          <t>AIA-CC-02</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>딥페이크·AI 사칭 기반 금전 사기</t>
-        </is>
-      </c>
-      <c r="D18" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+          <t>실행 중 AI 명령 동적 생성 악성코드</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>20</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>보조</t>
+          <t>반자율</t>
         </is>
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>증폭</t>
+          <t>신규</t>
         </is>
       </c>
       <c r="H18" s="9" t="inlineStr">
@@ -1561,88 +1561,92 @@
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>AI-01-08, ID-IM-01</t>
+          <t>AI-01-06</t>
         </is>
       </c>
       <c r="J18" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>[VE] 취약점 발굴·익스플로잇 생성</t>
+          <t>[CC] 은닉·명령제어</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>AIA-VE-01.1</t>
+          <t>AIA-CC-03</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>AI 자율 취약점 발굴(버그 헌팅)</t>
-        </is>
-      </c>
-      <c r="D19" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+          <t>AI 기반 방어 회피·난독화</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>23</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>완전자율</t>
+          <t>증강</t>
         </is>
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>신규</t>
+          <t>증폭</t>
         </is>
       </c>
       <c r="H19" s="9" t="inlineStr">
         <is>
-          <t>실사용</t>
-        </is>
-      </c>
-      <c r="I19" s="7" t="inlineStr"/>
+          <t>실증</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>AI-04-04</t>
+        </is>
+      </c>
       <c r="J19" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>[VE] 취약점 발굴·익스플로잇 생성</t>
+          <t>[CC] 은닉·명령제어</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>AIA-VE-02</t>
+          <t>AIA-CC-04</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>AI 익스플로잇 자동 생성·개발</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+          <t>AI 코딩 도구 규칙·설정 숨은 지시 주입</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>반자율</t>
+          <t>보조</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
@@ -1652,38 +1656,42 @@
       </c>
       <c r="H20" s="9" t="inlineStr">
         <is>
-          <t>실사용</t>
-        </is>
-      </c>
-      <c r="I20" s="7" t="inlineStr"/>
+          <t>실증</t>
+        </is>
+      </c>
+      <c r="I20" s="7" t="inlineStr">
+        <is>
+          <t>AI-08-05, SC-DE-02</t>
+        </is>
+      </c>
       <c r="J20" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>[VE] 취약점 발굴·익스플로잇 생성</t>
+          <t>[IA] 초기 침투·사회공학</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>AIA-VE-03.2</t>
+          <t>AIA-IA-01.1</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>AI 생성 와이퍼·파괴 스크립트</t>
-        </is>
-      </c>
-      <c r="D21" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+          <t>AI 생성 대량 피싱·미끼</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>13</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
@@ -1703,7 +1711,7 @@
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>AI-01-06, OT-IR-01</t>
+          <t>AI-01-08, ID-SE-01</t>
         </is>
       </c>
       <c r="J21" s="9" t="n">
@@ -1713,17 +1721,17 @@
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>[AO] 자율 실행·확산</t>
+          <t>[IA] 초기 침투·사회공학</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>AIA-AO-06</t>
+          <t>AIA-IA-01.2</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>통제를 벗어난 자율 에이전트의 자발적 침해(사람 공격자 없음)</t>
+          <t>AI 기반 표적 스피어피싱·BEC</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -1733,17 +1741,17 @@
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>29</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>완전자율</t>
+          <t>증강</t>
         </is>
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>신규</t>
+          <t>증폭</t>
         </is>
       </c>
       <c r="H22" s="9" t="inlineStr">
@@ -1753,27 +1761,27 @@
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>AI-01-05</t>
+          <t>AI-01-08, ID-SE-01</t>
         </is>
       </c>
       <c r="J22" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>[CC] 은닉·명령제어</t>
+          <t>[IA] 초기 침투·사회공학</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>AIA-CC-03</t>
+          <t>AIA-IA-02.2</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>AI 기반 방어 회피·난독화</t>
+          <t>음성 딥페이크 사칭</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
@@ -1783,12 +1791,12 @@
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>15</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>증강</t>
+          <t>보조</t>
         </is>
       </c>
       <c r="G23" s="9" t="inlineStr">
@@ -1798,32 +1806,32 @@
       </c>
       <c r="H23" s="9" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>실사용</t>
         </is>
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>AI-04-04</t>
+          <t>AI-01-08, ID-SE-04</t>
         </is>
       </c>
       <c r="J23" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>[CC] 은닉·명령제어</t>
+          <t>[IA] 초기 침투·사회공학</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>AIA-CC-04</t>
+          <t>AIA-IA-04</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>AI 코딩 도구 규칙·설정 숨은 지시 주입</t>
+          <t>AI 미끼·ClickFix·크래프트 링크로 실행 유도</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -1833,7 +1841,7 @@
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
@@ -1853,27 +1861,27 @@
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>AI-08-05, SC-DE-02</t>
+          <t>AI-01-08</t>
         </is>
       </c>
       <c r="J24" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>[IA] 초기 침투·사회공학</t>
+          <t>[IM] 영향·규모화</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>AIA-IA-01.2</t>
+          <t>AIA-IM-04</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>AI 기반 표적 스피어피싱·BEC</t>
+          <t>AI 활용 공격의 규모화·대량화</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
@@ -1883,12 +1891,12 @@
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>28</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>증강</t>
+          <t>반자율</t>
         </is>
       </c>
       <c r="G25" s="9" t="inlineStr">
@@ -1903,27 +1911,27 @@
       </c>
       <c r="I25" s="7" t="inlineStr">
         <is>
-          <t>AI-01-08, ID-SE-01</t>
+          <t>AI-01-05</t>
         </is>
       </c>
       <c r="J25" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>[IA] 초기 침투·사회공학</t>
+          <t>[RD] 공격 역량 확보</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>AIA-IA-02.2</t>
+          <t>AIA-RD-01.1</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>음성 딥페이크 사칭</t>
+          <t>다크 LLM·탈옥 모델 확보</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -1933,7 +1941,7 @@
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>26</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
@@ -1943,7 +1951,7 @@
       </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>증폭</t>
+          <t>신규</t>
         </is>
       </c>
       <c r="H26" s="9" t="inlineStr">
@@ -1953,27 +1961,27 @@
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>AI-01-08, ID-SE-04</t>
+          <t>AI-01-03</t>
         </is>
       </c>
       <c r="J26" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>[IA] 초기 침투·사회공학</t>
+          <t>[RD] 공격 역량 확보</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>AIA-IA-04</t>
+          <t>AIA-RD-02</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>AI 미끼·ClickFix·크래프트 링크로 실행 유도</t>
+          <t>AI 기반 공격 도구·스크립트·셸 명령 생성</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
@@ -1988,22 +1996,22 @@
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>보조</t>
+          <t>증강</t>
         </is>
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t>신규</t>
+          <t>증폭</t>
         </is>
       </c>
       <c r="H27" s="9" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>실사용</t>
         </is>
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>AI-01-08</t>
+          <t>AI-01-03</t>
         </is>
       </c>
       <c r="J27" s="9" t="n">
@@ -2013,17 +2021,17 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>[IM] 영향·규모화</t>
+          <t>[RD] 공격 역량 확보</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>AIA-IM-04</t>
+          <t>AIA-RD-03</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>AI 활용 공격의 규모화·대량화</t>
+          <t>공격 인프라·AI 서비스 프록시 확보</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2033,12 +2041,12 @@
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>반자율</t>
+          <t>보조</t>
         </is>
       </c>
       <c r="G28" s="9" t="inlineStr">
@@ -2048,32 +2056,32 @@
       </c>
       <c r="H28" s="9" t="inlineStr">
         <is>
-          <t>실사용</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>AI-01-05</t>
+          <t>AI-09-03, CL-RD-01</t>
         </is>
       </c>
       <c r="J28" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>[RD] 공격 역량 확보</t>
+          <t>[RT] 정찰·표적 분석</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>AIA-RD-01.1</t>
+          <t>AIA-RT-01.1</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>다크 LLM·탈옥 모델 확보</t>
+          <t>AI 기반 공개정보 수집·인물 프로파일링</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
@@ -2083,17 +2091,17 @@
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>25</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>보조</t>
+          <t>증강</t>
         </is>
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>신규</t>
+          <t>증폭</t>
         </is>
       </c>
       <c r="H29" s="9" t="inlineStr">
@@ -2103,27 +2111,27 @@
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>AI-01-03</t>
+          <t>AI-01-01, PH-RC-01</t>
         </is>
       </c>
       <c r="J29" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>[RD] 공격 역량 확보</t>
+          <t>[RT] 정찰·표적 분석</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>AIA-RD-02</t>
+          <t>AIA-RT-01.2</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>AI 기반 공격 도구·스크립트·셸 명령 생성</t>
+          <t>AI 기반 표적 환경·관계 분석</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2133,7 +2141,7 @@
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
@@ -2148,12 +2156,12 @@
       </c>
       <c r="H30" s="9" t="inlineStr">
         <is>
-          <t>실사용</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>AI-01-03</t>
+          <t>AI-01-01</t>
         </is>
       </c>
       <c r="J30" s="9" t="n">
@@ -2163,17 +2171,17 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>[RD] 공격 역량 확보</t>
+          <t>[RT] 정찰·표적 분석</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>AIA-RD-03</t>
+          <t>AIA-RT-02</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>공격 인프라·AI 서비스 프록시 확보</t>
+          <t>AI 에이전트의 노출 자산·공격면 자동 식별</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr">
@@ -2183,12 +2191,12 @@
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>14</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>보조</t>
+          <t>반자율</t>
         </is>
       </c>
       <c r="G31" s="9" t="inlineStr">
@@ -2198,16 +2206,16 @@
       </c>
       <c r="H31" s="9" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>실사용</t>
         </is>
       </c>
       <c r="I31" s="7" t="inlineStr">
         <is>
-          <t>AI-09-03, CL-RD-01</t>
+          <t>AI-01-01</t>
         </is>
       </c>
       <c r="J31" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -2218,12 +2226,12 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>AIA-RT-01.1</t>
+          <t>AIA-RT-03</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>AI 기반 공개정보 수집·인물 프로파일링</t>
+          <t>AI 기반 취약점 정보·공개 PoC 자동 수집·분류</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2233,7 +2241,7 @@
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>18</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
@@ -2253,27 +2261,27 @@
       </c>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t>AI-01-01, PH-RC-01</t>
+          <t>AI-01-03</t>
         </is>
       </c>
       <c r="J32" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>[RT] 정찰·표적 분석</t>
+          <t>[VE] 취약점 발굴·익스플로잇 생성</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>AIA-RT-01.2</t>
+          <t>AIA-VE-01.1</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>AI 기반 표적 환경·관계 분석</t>
+          <t>AI 자율 취약점 발굴(버그 헌팅)</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr">
@@ -2283,47 +2291,43 @@
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>증강</t>
+          <t>완전자율</t>
         </is>
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
-          <t>증폭</t>
+          <t>신규</t>
         </is>
       </c>
       <c r="H33" s="9" t="inlineStr">
         <is>
-          <t>실증</t>
-        </is>
-      </c>
-      <c r="I33" s="7" t="inlineStr">
-        <is>
-          <t>AI-01-01</t>
-        </is>
-      </c>
+          <t>실사용</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="inlineStr"/>
       <c r="J33" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>[RT] 정찰·표적 분석</t>
+          <t>[VE] 취약점 발굴·익스플로잇 생성</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>AIA-RT-02</t>
+          <t>AIA-VE-01.2</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>AI 에이전트의 노출 자산·공격면 자동 식별</t>
+          <t>AI 보조 코드 감사·퍼징</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2333,12 +2337,12 @@
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>32</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>반자율</t>
+          <t>증강</t>
         </is>
       </c>
       <c r="G34" s="9" t="inlineStr">
@@ -2348,12 +2352,12 @@
       </c>
       <c r="H34" s="9" t="inlineStr">
         <is>
-          <t>실사용</t>
+          <t>실증</t>
         </is>
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>AI-01-01</t>
+          <t>SC-DP-04</t>
         </is>
       </c>
       <c r="J34" s="9" t="n">
@@ -2363,17 +2367,17 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>[RT] 정찰·표적 분석</t>
+          <t>[VE] 취약점 발굴·익스플로잇 생성</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>AIA-RT-03</t>
+          <t>AIA-VE-02</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>AI 기반 취약점 정보·공개 PoC 자동 수집·분류</t>
+          <t>AI 익스플로잇 자동 생성·개발</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
@@ -2383,17 +2387,17 @@
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>33</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>증강</t>
+          <t>반자율</t>
         </is>
       </c>
       <c r="G35" s="9" t="inlineStr">
         <is>
-          <t>증폭</t>
+          <t>신규</t>
         </is>
       </c>
       <c r="H35" s="9" t="inlineStr">
@@ -2401,13 +2405,9 @@
           <t>실사용</t>
         </is>
       </c>
-      <c r="I35" s="7" t="inlineStr">
-        <is>
-          <t>AI-01-03</t>
-        </is>
-      </c>
+      <c r="I35" s="7" t="inlineStr"/>
       <c r="J35" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -2418,12 +2418,12 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>AIA-VE-01.2</t>
+          <t>AIA-VE-03.2</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>AI 보조 코드 감사·퍼징</t>
+          <t>AI 생성 와이퍼·파괴 스크립트</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -2433,12 +2433,12 @@
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>16</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>증강</t>
+          <t>보조</t>
         </is>
       </c>
       <c r="G36" s="9" t="inlineStr">
@@ -2448,16 +2448,16 @@
       </c>
       <c r="H36" s="9" t="inlineStr">
         <is>
-          <t>실증</t>
+          <t>실사용</t>
         </is>
       </c>
       <c r="I36" s="7" t="inlineStr">
         <is>
-          <t>SC-DP-04</t>
+          <t>AI-01-06, OT-IR-01</t>
         </is>
       </c>
       <c r="J36" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
@@ -3033,9 +3033,9 @@
           <t>AI 서비스 API·웹 인터페이스 경유 은닉 C2</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -3070,9 +3070,9 @@
           <t>실행 중 AI 명령 동적 생성 악성코드</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -3218,9 +3218,9 @@
           <t>AI 생성 대량 피싱·미끼</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -3255,9 +3255,9 @@
           <t>AI 생성 대량 피싱·미끼</t>
         </is>
       </c>
-      <c r="C22" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -3995,9 +3995,9 @@
           <t>공세 AI 에이전트·공격 하네스 구축</t>
         </is>
       </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>매우 높음</t>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>높음</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
@@ -4254,9 +4254,9 @@
           <t>AI 생성·AI 연동 악성코드</t>
         </is>
       </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>매우 높음</t>
+      <c r="C49" s="10" t="inlineStr">
+        <is>
+          <t>높음</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
@@ -4291,9 +4291,9 @@
           <t>AI 생성 와이퍼·파괴 스크립트</t>
         </is>
       </c>
-      <c r="C50" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+      <c r="C50" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
@@ -4328,9 +4328,9 @@
           <t>AI 생성 와이퍼·파괴 스크립트</t>
         </is>
       </c>
-      <c r="C51" s="10" t="inlineStr">
-        <is>
-          <t>높음</t>
+      <c r="C51" s="11" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">

</xml_diff>